<commit_message>
feat: Cap nhat cot LOAI_THUOC mac dinh bang 3 cho Vat Tu Y Te
</commit_message>
<xml_diff>
--- a/data/File_Import_VTYT_VNPT_HIS_78cot.xlsx
+++ b/data/File_Import_VTYT_VNPT_HIS_78cot.xlsx
@@ -768,8 +768,8 @@
       <c r="AR2">
         <v>11055</v>
       </c>
-      <c r="AS2" t="str">
-        <v/>
+      <c r="AS2">
+        <v>3</v>
       </c>
       <c r="AT2">
         <v>2</v>
@@ -1004,8 +1004,8 @@
       <c r="AR3">
         <v>11055</v>
       </c>
-      <c r="AS3" t="str">
-        <v/>
+      <c r="AS3">
+        <v>3</v>
       </c>
       <c r="AT3">
         <v>2</v>
@@ -1240,8 +1240,8 @@
       <c r="AR4">
         <v>11055</v>
       </c>
-      <c r="AS4" t="str">
-        <v/>
+      <c r="AS4">
+        <v>3</v>
       </c>
       <c r="AT4">
         <v>2</v>
@@ -1476,8 +1476,8 @@
       <c r="AR5">
         <v>11055</v>
       </c>
-      <c r="AS5" t="str">
-        <v/>
+      <c r="AS5">
+        <v>3</v>
       </c>
       <c r="AT5">
         <v>2</v>
@@ -1712,8 +1712,8 @@
       <c r="AR6">
         <v>11055</v>
       </c>
-      <c r="AS6" t="str">
-        <v/>
+      <c r="AS6">
+        <v>3</v>
       </c>
       <c r="AT6">
         <v>2</v>
@@ -1948,8 +1948,8 @@
       <c r="AR7">
         <v>11055</v>
       </c>
-      <c r="AS7" t="str">
-        <v/>
+      <c r="AS7">
+        <v>3</v>
       </c>
       <c r="AT7">
         <v>2</v>
@@ -2184,8 +2184,8 @@
       <c r="AR8">
         <v>11055</v>
       </c>
-      <c r="AS8" t="str">
-        <v/>
+      <c r="AS8">
+        <v>3</v>
       </c>
       <c r="AT8">
         <v>2</v>
@@ -2420,8 +2420,8 @@
       <c r="AR9">
         <v>11055</v>
       </c>
-      <c r="AS9" t="str">
-        <v/>
+      <c r="AS9">
+        <v>3</v>
       </c>
       <c r="AT9">
         <v>2</v>
@@ -2656,8 +2656,8 @@
       <c r="AR10">
         <v>11055</v>
       </c>
-      <c r="AS10" t="str">
-        <v/>
+      <c r="AS10">
+        <v>3</v>
       </c>
       <c r="AT10">
         <v>2</v>
@@ -2892,8 +2892,8 @@
       <c r="AR11">
         <v>11055</v>
       </c>
-      <c r="AS11" t="str">
-        <v/>
+      <c r="AS11">
+        <v>3</v>
       </c>
       <c r="AT11">
         <v>2</v>
@@ -3128,8 +3128,8 @@
       <c r="AR12">
         <v>11055</v>
       </c>
-      <c r="AS12" t="str">
-        <v/>
+      <c r="AS12">
+        <v>3</v>
       </c>
       <c r="AT12">
         <v>2</v>
@@ -3364,8 +3364,8 @@
       <c r="AR13">
         <v>11055</v>
       </c>
-      <c r="AS13" t="str">
-        <v/>
+      <c r="AS13">
+        <v>3</v>
       </c>
       <c r="AT13">
         <v>2</v>
@@ -3600,8 +3600,8 @@
       <c r="AR14">
         <v>11055</v>
       </c>
-      <c r="AS14" t="str">
-        <v/>
+      <c r="AS14">
+        <v>3</v>
       </c>
       <c r="AT14">
         <v>2</v>
@@ -3836,8 +3836,8 @@
       <c r="AR15">
         <v>11055</v>
       </c>
-      <c r="AS15" t="str">
-        <v/>
+      <c r="AS15">
+        <v>3</v>
       </c>
       <c r="AT15">
         <v>2</v>
@@ -4072,8 +4072,8 @@
       <c r="AR16">
         <v>11055</v>
       </c>
-      <c r="AS16" t="str">
-        <v/>
+      <c r="AS16">
+        <v>3</v>
       </c>
       <c r="AT16">
         <v>2</v>
@@ -4308,8 +4308,8 @@
       <c r="AR17">
         <v>11055</v>
       </c>
-      <c r="AS17" t="str">
-        <v/>
+      <c r="AS17">
+        <v>3</v>
       </c>
       <c r="AT17">
         <v>2</v>
@@ -4544,8 +4544,8 @@
       <c r="AR18">
         <v>11055</v>
       </c>
-      <c r="AS18" t="str">
-        <v/>
+      <c r="AS18">
+        <v>3</v>
       </c>
       <c r="AT18">
         <v>2</v>
@@ -4780,8 +4780,8 @@
       <c r="AR19">
         <v>11055</v>
       </c>
-      <c r="AS19" t="str">
-        <v/>
+      <c r="AS19">
+        <v>3</v>
       </c>
       <c r="AT19">
         <v>2</v>
@@ -5016,8 +5016,8 @@
       <c r="AR20">
         <v>11055</v>
       </c>
-      <c r="AS20" t="str">
-        <v/>
+      <c r="AS20">
+        <v>3</v>
       </c>
       <c r="AT20">
         <v>2</v>
@@ -5252,8 +5252,8 @@
       <c r="AR21">
         <v>11055</v>
       </c>
-      <c r="AS21" t="str">
-        <v/>
+      <c r="AS21">
+        <v>3</v>
       </c>
       <c r="AT21">
         <v>2</v>
@@ -5488,8 +5488,8 @@
       <c r="AR22">
         <v>11055</v>
       </c>
-      <c r="AS22" t="str">
-        <v/>
+      <c r="AS22">
+        <v>3</v>
       </c>
       <c r="AT22">
         <v>2</v>
@@ -5724,8 +5724,8 @@
       <c r="AR23">
         <v>11055</v>
       </c>
-      <c r="AS23" t="str">
-        <v/>
+      <c r="AS23">
+        <v>3</v>
       </c>
       <c r="AT23">
         <v>2</v>
@@ -5960,8 +5960,8 @@
       <c r="AR24">
         <v>11055</v>
       </c>
-      <c r="AS24" t="str">
-        <v/>
+      <c r="AS24">
+        <v>3</v>
       </c>
       <c r="AT24">
         <v>2</v>
@@ -6196,8 +6196,8 @@
       <c r="AR25">
         <v>11055</v>
       </c>
-      <c r="AS25" t="str">
-        <v/>
+      <c r="AS25">
+        <v>3</v>
       </c>
       <c r="AT25">
         <v>2</v>
@@ -6432,8 +6432,8 @@
       <c r="AR26">
         <v>11055</v>
       </c>
-      <c r="AS26" t="str">
-        <v/>
+      <c r="AS26">
+        <v>3</v>
       </c>
       <c r="AT26">
         <v>2</v>
@@ -6668,8 +6668,8 @@
       <c r="AR27">
         <v>11055</v>
       </c>
-      <c r="AS27" t="str">
-        <v/>
+      <c r="AS27">
+        <v>3</v>
       </c>
       <c r="AT27">
         <v>2</v>
@@ -6904,8 +6904,8 @@
       <c r="AR28">
         <v>11055</v>
       </c>
-      <c r="AS28" t="str">
-        <v/>
+      <c r="AS28">
+        <v>3</v>
       </c>
       <c r="AT28">
         <v>2</v>
@@ -7140,8 +7140,8 @@
       <c r="AR29">
         <v>11055</v>
       </c>
-      <c r="AS29" t="str">
-        <v/>
+      <c r="AS29">
+        <v>3</v>
       </c>
       <c r="AT29">
         <v>2</v>
@@ -7376,8 +7376,8 @@
       <c r="AR30">
         <v>11055</v>
       </c>
-      <c r="AS30" t="str">
-        <v/>
+      <c r="AS30">
+        <v>3</v>
       </c>
       <c r="AT30">
         <v>2</v>
@@ -7612,8 +7612,8 @@
       <c r="AR31">
         <v>11055</v>
       </c>
-      <c r="AS31" t="str">
-        <v/>
+      <c r="AS31">
+        <v>3</v>
       </c>
       <c r="AT31">
         <v>2</v>
@@ -7850,8 +7850,8 @@
       <c r="AR32">
         <v>11055</v>
       </c>
-      <c r="AS32" t="str">
-        <v/>
+      <c r="AS32">
+        <v>3</v>
       </c>
       <c r="AT32">
         <v>2</v>
@@ -8086,8 +8086,8 @@
       <c r="AR33">
         <v>11055</v>
       </c>
-      <c r="AS33" t="str">
-        <v/>
+      <c r="AS33">
+        <v>3</v>
       </c>
       <c r="AT33">
         <v>2</v>
@@ -8322,8 +8322,8 @@
       <c r="AR34">
         <v>11055</v>
       </c>
-      <c r="AS34" t="str">
-        <v/>
+      <c r="AS34">
+        <v>3</v>
       </c>
       <c r="AT34">
         <v>2</v>
@@ -8558,8 +8558,8 @@
       <c r="AR35">
         <v>11055</v>
       </c>
-      <c r="AS35" t="str">
-        <v/>
+      <c r="AS35">
+        <v>3</v>
       </c>
       <c r="AT35">
         <v>2</v>
@@ -8794,8 +8794,8 @@
       <c r="AR36">
         <v>11055</v>
       </c>
-      <c r="AS36" t="str">
-        <v/>
+      <c r="AS36">
+        <v>3</v>
       </c>
       <c r="AT36">
         <v>2</v>
@@ -9030,8 +9030,8 @@
       <c r="AR37">
         <v>11055</v>
       </c>
-      <c r="AS37" t="str">
-        <v/>
+      <c r="AS37">
+        <v>3</v>
       </c>
       <c r="AT37">
         <v>2</v>
@@ -9266,8 +9266,8 @@
       <c r="AR38">
         <v>11055</v>
       </c>
-      <c r="AS38" t="str">
-        <v/>
+      <c r="AS38">
+        <v>3</v>
       </c>
       <c r="AT38">
         <v>2</v>
@@ -9502,8 +9502,8 @@
       <c r="AR39">
         <v>11055</v>
       </c>
-      <c r="AS39" t="str">
-        <v/>
+      <c r="AS39">
+        <v>3</v>
       </c>
       <c r="AT39">
         <v>2</v>
@@ -9738,8 +9738,8 @@
       <c r="AR40">
         <v>11055</v>
       </c>
-      <c r="AS40" t="str">
-        <v/>
+      <c r="AS40">
+        <v>3</v>
       </c>
       <c r="AT40">
         <v>2</v>
@@ -9974,8 +9974,8 @@
       <c r="AR41">
         <v>11055</v>
       </c>
-      <c r="AS41" t="str">
-        <v/>
+      <c r="AS41">
+        <v>3</v>
       </c>
       <c r="AT41">
         <v>2</v>
@@ -10210,8 +10210,8 @@
       <c r="AR42">
         <v>11055</v>
       </c>
-      <c r="AS42" t="str">
-        <v/>
+      <c r="AS42">
+        <v>3</v>
       </c>
       <c r="AT42">
         <v>2</v>
@@ -10446,8 +10446,8 @@
       <c r="AR43">
         <v>11055</v>
       </c>
-      <c r="AS43" t="str">
-        <v/>
+      <c r="AS43">
+        <v>3</v>
       </c>
       <c r="AT43">
         <v>2</v>
@@ -10682,8 +10682,8 @@
       <c r="AR44">
         <v>11055</v>
       </c>
-      <c r="AS44" t="str">
-        <v/>
+      <c r="AS44">
+        <v>3</v>
       </c>
       <c r="AT44">
         <v>2</v>
@@ -10918,8 +10918,8 @@
       <c r="AR45">
         <v>11055</v>
       </c>
-      <c r="AS45" t="str">
-        <v/>
+      <c r="AS45">
+        <v>3</v>
       </c>
       <c r="AT45">
         <v>2</v>
@@ -11154,8 +11154,8 @@
       <c r="AR46">
         <v>11055</v>
       </c>
-      <c r="AS46" t="str">
-        <v/>
+      <c r="AS46">
+        <v>3</v>
       </c>
       <c r="AT46">
         <v>2</v>

</xml_diff>

<commit_message>
feat: Bo tran bao hiem GIA_BHYT_QUYET_TOAN (de trong) o Tab Gen File Thuoc va Vat Tu
</commit_message>
<xml_diff>
--- a/data/File_Import_VTYT_VNPT_HIS_78cot.xlsx
+++ b/data/File_Import_VTYT_VNPT_HIS_78cot.xlsx
@@ -679,7 +679,7 @@
         <v>777</v>
       </c>
       <c r="O2">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P2">
         <v>777</v>
@@ -690,8 +690,8 @@
       <c r="R2">
         <v>777</v>
       </c>
-      <c r="S2">
-        <v>777</v>
+      <c r="S2" t="str">
+        <v/>
       </c>
       <c r="T2">
         <v>100</v>
@@ -915,7 +915,7 @@
         <v>1260</v>
       </c>
       <c r="O3">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P3">
         <v>1260</v>
@@ -926,8 +926,8 @@
       <c r="R3">
         <v>1260</v>
       </c>
-      <c r="S3">
-        <v>1260</v>
+      <c r="S3" t="str">
+        <v/>
       </c>
       <c r="T3">
         <v>100</v>
@@ -1151,7 +1151,7 @@
         <v>5481</v>
       </c>
       <c r="O4">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P4">
         <v>5481</v>
@@ -1162,8 +1162,8 @@
       <c r="R4">
         <v>5481</v>
       </c>
-      <c r="S4">
-        <v>5481</v>
+      <c r="S4" t="str">
+        <v/>
       </c>
       <c r="T4">
         <v>100</v>
@@ -1387,7 +1387,7 @@
         <v>420</v>
       </c>
       <c r="O5">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P5">
         <v>420</v>
@@ -1398,8 +1398,8 @@
       <c r="R5">
         <v>420</v>
       </c>
-      <c r="S5">
-        <v>420</v>
+      <c r="S5" t="str">
+        <v/>
       </c>
       <c r="T5">
         <v>100</v>
@@ -1623,7 +1623,7 @@
         <v>1260</v>
       </c>
       <c r="O6">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P6">
         <v>1260</v>
@@ -1634,8 +1634,8 @@
       <c r="R6">
         <v>1260</v>
       </c>
-      <c r="S6">
-        <v>1260</v>
+      <c r="S6" t="str">
+        <v/>
       </c>
       <c r="T6">
         <v>100</v>
@@ -1859,7 +1859,7 @@
         <v>777</v>
       </c>
       <c r="O7">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P7">
         <v>777</v>
@@ -1870,8 +1870,8 @@
       <c r="R7">
         <v>777</v>
       </c>
-      <c r="S7">
-        <v>777</v>
+      <c r="S7" t="str">
+        <v/>
       </c>
       <c r="T7">
         <v>100</v>
@@ -2095,7 +2095,7 @@
         <v>2205</v>
       </c>
       <c r="O8">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P8">
         <v>2205</v>
@@ -2106,8 +2106,8 @@
       <c r="R8">
         <v>2205</v>
       </c>
-      <c r="S8">
-        <v>2205</v>
+      <c r="S8" t="str">
+        <v/>
       </c>
       <c r="T8">
         <v>100</v>
@@ -2331,7 +2331,7 @@
         <v>5481</v>
       </c>
       <c r="O9">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P9">
         <v>5481</v>
@@ -2342,8 +2342,8 @@
       <c r="R9">
         <v>5481</v>
       </c>
-      <c r="S9">
-        <v>5481</v>
+      <c r="S9" t="str">
+        <v/>
       </c>
       <c r="T9">
         <v>100</v>
@@ -2567,7 +2567,7 @@
         <v>777</v>
       </c>
       <c r="O10">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P10">
         <v>777</v>
@@ -2578,8 +2578,8 @@
       <c r="R10">
         <v>777</v>
       </c>
-      <c r="S10">
-        <v>777</v>
+      <c r="S10" t="str">
+        <v/>
       </c>
       <c r="T10">
         <v>100</v>
@@ -2803,7 +2803,7 @@
         <v>5481</v>
       </c>
       <c r="O11">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P11">
         <v>5481</v>
@@ -2814,8 +2814,8 @@
       <c r="R11">
         <v>5481</v>
       </c>
-      <c r="S11">
-        <v>5481</v>
+      <c r="S11" t="str">
+        <v/>
       </c>
       <c r="T11">
         <v>100</v>
@@ -3039,7 +3039,7 @@
         <v>420</v>
       </c>
       <c r="O12">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P12">
         <v>420</v>
@@ -3050,8 +3050,8 @@
       <c r="R12">
         <v>420</v>
       </c>
-      <c r="S12">
-        <v>420</v>
+      <c r="S12" t="str">
+        <v/>
       </c>
       <c r="T12">
         <v>100</v>
@@ -3275,7 +3275,7 @@
         <v>1260</v>
       </c>
       <c r="O13">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P13">
         <v>1260</v>
@@ -3286,8 +3286,8 @@
       <c r="R13">
         <v>1260</v>
       </c>
-      <c r="S13">
-        <v>1260</v>
+      <c r="S13" t="str">
+        <v/>
       </c>
       <c r="T13">
         <v>100</v>
@@ -3511,7 +3511,7 @@
         <v>9996</v>
       </c>
       <c r="O14">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P14">
         <v>9996</v>
@@ -3522,8 +3522,8 @@
       <c r="R14">
         <v>9996</v>
       </c>
-      <c r="S14">
-        <v>9996</v>
+      <c r="S14" t="str">
+        <v/>
       </c>
       <c r="T14">
         <v>100</v>
@@ -3747,7 +3747,7 @@
         <v>1155</v>
       </c>
       <c r="O15">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P15">
         <v>1155</v>
@@ -3758,8 +3758,8 @@
       <c r="R15">
         <v>1155</v>
       </c>
-      <c r="S15">
-        <v>1155</v>
+      <c r="S15" t="str">
+        <v/>
       </c>
       <c r="T15">
         <v>100</v>
@@ -3983,7 +3983,7 @@
         <v>714</v>
       </c>
       <c r="O16">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P16">
         <v>714</v>
@@ -3994,8 +3994,8 @@
       <c r="R16">
         <v>714</v>
       </c>
-      <c r="S16">
-        <v>714</v>
+      <c r="S16" t="str">
+        <v/>
       </c>
       <c r="T16">
         <v>100</v>
@@ -4219,7 +4219,7 @@
         <v>2100</v>
       </c>
       <c r="O17">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P17">
         <v>2100</v>
@@ -4230,8 +4230,8 @@
       <c r="R17">
         <v>2100</v>
       </c>
-      <c r="S17">
-        <v>2100</v>
+      <c r="S17" t="str">
+        <v/>
       </c>
       <c r="T17">
         <v>100</v>
@@ -4455,7 +4455,7 @@
         <v>749.7</v>
       </c>
       <c r="O18">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P18">
         <v>749.7</v>
@@ -4466,8 +4466,8 @@
       <c r="R18">
         <v>749.7</v>
       </c>
-      <c r="S18">
-        <v>749.7</v>
+      <c r="S18" t="str">
+        <v/>
       </c>
       <c r="T18">
         <v>100</v>
@@ -4691,7 +4691,7 @@
         <v>4494</v>
       </c>
       <c r="O19">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P19">
         <v>4494</v>
@@ -4702,8 +4702,8 @@
       <c r="R19">
         <v>4494</v>
       </c>
-      <c r="S19">
-        <v>4494</v>
+      <c r="S19" t="str">
+        <v/>
       </c>
       <c r="T19">
         <v>100</v>
@@ -4927,7 +4927,7 @@
         <v>15000</v>
       </c>
       <c r="O20">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P20">
         <v>15000</v>
@@ -4938,8 +4938,8 @@
       <c r="R20">
         <v>15000</v>
       </c>
-      <c r="S20">
-        <v>15000</v>
+      <c r="S20" t="str">
+        <v/>
       </c>
       <c r="T20">
         <v>100</v>
@@ -5163,7 +5163,7 @@
         <v>357</v>
       </c>
       <c r="O21">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P21">
         <v>357</v>
@@ -5174,8 +5174,8 @@
       <c r="R21">
         <v>357</v>
       </c>
-      <c r="S21">
-        <v>357</v>
+      <c r="S21" t="str">
+        <v/>
       </c>
       <c r="T21">
         <v>100</v>
@@ -5399,7 +5399,7 @@
         <v>1134</v>
       </c>
       <c r="O22">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P22">
         <v>1134</v>
@@ -5410,8 +5410,8 @@
       <c r="R22">
         <v>1134</v>
       </c>
-      <c r="S22">
-        <v>1134</v>
+      <c r="S22" t="str">
+        <v/>
       </c>
       <c r="T22">
         <v>100</v>
@@ -5635,7 +5635,7 @@
         <v>5250</v>
       </c>
       <c r="O23">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P23">
         <v>5250</v>
@@ -5646,8 +5646,8 @@
       <c r="R23">
         <v>5250</v>
       </c>
-      <c r="S23">
-        <v>5250</v>
+      <c r="S23" t="str">
+        <v/>
       </c>
       <c r="T23">
         <v>100</v>
@@ -5871,7 +5871,7 @@
         <v>5460</v>
       </c>
       <c r="O24">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P24">
         <v>5460</v>
@@ -5882,8 +5882,8 @@
       <c r="R24">
         <v>5460</v>
       </c>
-      <c r="S24">
-        <v>5460</v>
+      <c r="S24" t="str">
+        <v/>
       </c>
       <c r="T24">
         <v>100</v>
@@ -6107,7 +6107,7 @@
         <v>18800</v>
       </c>
       <c r="O25">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P25">
         <v>18800</v>
@@ -6118,8 +6118,8 @@
       <c r="R25">
         <v>18800</v>
       </c>
-      <c r="S25">
-        <v>18800</v>
+      <c r="S25" t="str">
+        <v/>
       </c>
       <c r="T25">
         <v>100</v>
@@ -6343,7 +6343,7 @@
         <v>12500</v>
       </c>
       <c r="O26">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P26">
         <v>12500</v>
@@ -6354,8 +6354,8 @@
       <c r="R26">
         <v>12500</v>
       </c>
-      <c r="S26">
-        <v>12500</v>
+      <c r="S26" t="str">
+        <v/>
       </c>
       <c r="T26">
         <v>100</v>
@@ -6579,7 +6579,7 @@
         <v>15800</v>
       </c>
       <c r="O27">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P27">
         <v>15800</v>
@@ -6590,8 +6590,8 @@
       <c r="R27">
         <v>15800</v>
       </c>
-      <c r="S27">
-        <v>15800</v>
+      <c r="S27" t="str">
+        <v/>
       </c>
       <c r="T27">
         <v>100</v>
@@ -6815,7 +6815,7 @@
         <v>6100</v>
       </c>
       <c r="O28">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P28">
         <v>6100</v>
@@ -6826,8 +6826,8 @@
       <c r="R28">
         <v>6100</v>
       </c>
-      <c r="S28">
-        <v>6100</v>
+      <c r="S28" t="str">
+        <v/>
       </c>
       <c r="T28">
         <v>100</v>
@@ -7051,7 +7051,7 @@
         <v>15000</v>
       </c>
       <c r="O29">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P29">
         <v>15000</v>
@@ -7062,8 +7062,8 @@
       <c r="R29">
         <v>15000</v>
       </c>
-      <c r="S29">
-        <v>15000</v>
+      <c r="S29" t="str">
+        <v/>
       </c>
       <c r="T29">
         <v>100</v>
@@ -7287,7 +7287,7 @@
         <v>16000</v>
       </c>
       <c r="O30">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P30">
         <v>16000</v>
@@ -7298,8 +7298,8 @@
       <c r="R30">
         <v>16000</v>
       </c>
-      <c r="S30">
-        <v>16000</v>
+      <c r="S30" t="str">
+        <v/>
       </c>
       <c r="T30">
         <v>100</v>
@@ -7523,7 +7523,7 @@
         <v>12000</v>
       </c>
       <c r="O31">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P31">
         <v>12000</v>
@@ -7534,8 +7534,8 @@
       <c r="R31">
         <v>12000</v>
       </c>
-      <c r="S31">
-        <v>12000</v>
+      <c r="S31" t="str">
+        <v/>
       </c>
       <c r="T31">
         <v>100</v>
@@ -7759,7 +7759,7 @@
         <v>15700</v>
       </c>
       <c r="O32">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P32">
         <v>15700</v>
@@ -7770,8 +7770,8 @@
       <c r="R32">
         <v>15700</v>
       </c>
-      <c r="S32">
-        <v>15700</v>
+      <c r="S32" t="str">
+        <v/>
       </c>
       <c r="T32">
         <v>100</v>
@@ -7997,7 +7997,7 @@
         <v>16000</v>
       </c>
       <c r="O33">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P33">
         <v>16000</v>
@@ -8008,8 +8008,8 @@
       <c r="R33">
         <v>16000</v>
       </c>
-      <c r="S33">
-        <v>16000</v>
+      <c r="S33" t="str">
+        <v/>
       </c>
       <c r="T33">
         <v>100</v>
@@ -8233,7 +8233,7 @@
         <v>6000</v>
       </c>
       <c r="O34">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P34">
         <v>6000</v>
@@ -8244,8 +8244,8 @@
       <c r="R34">
         <v>6000</v>
       </c>
-      <c r="S34">
-        <v>6000</v>
+      <c r="S34" t="str">
+        <v/>
       </c>
       <c r="T34">
         <v>100</v>
@@ -8469,7 +8469,7 @@
         <v>15000</v>
       </c>
       <c r="O35">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P35">
         <v>15000</v>
@@ -8480,8 +8480,8 @@
       <c r="R35">
         <v>15000</v>
       </c>
-      <c r="S35">
-        <v>15000</v>
+      <c r="S35" t="str">
+        <v/>
       </c>
       <c r="T35">
         <v>100</v>
@@ -8705,7 +8705,7 @@
         <v>5481</v>
       </c>
       <c r="O36">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P36">
         <v>5481</v>
@@ -8716,8 +8716,8 @@
       <c r="R36">
         <v>5481</v>
       </c>
-      <c r="S36">
-        <v>5481</v>
+      <c r="S36" t="str">
+        <v/>
       </c>
       <c r="T36">
         <v>100</v>
@@ -8941,7 +8941,7 @@
         <v>1260</v>
       </c>
       <c r="O37">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P37">
         <v>1260</v>
@@ -8952,8 +8952,8 @@
       <c r="R37">
         <v>1260</v>
       </c>
-      <c r="S37">
-        <v>1260</v>
+      <c r="S37" t="str">
+        <v/>
       </c>
       <c r="T37">
         <v>100</v>
@@ -9177,7 +9177,7 @@
         <v>777</v>
       </c>
       <c r="O38">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P38">
         <v>777</v>
@@ -9188,8 +9188,8 @@
       <c r="R38">
         <v>777</v>
       </c>
-      <c r="S38">
-        <v>777</v>
+      <c r="S38" t="str">
+        <v/>
       </c>
       <c r="T38">
         <v>100</v>
@@ -9413,7 +9413,7 @@
         <v>2205</v>
       </c>
       <c r="O39">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P39">
         <v>2205</v>
@@ -9424,8 +9424,8 @@
       <c r="R39">
         <v>2205</v>
       </c>
-      <c r="S39">
-        <v>2205</v>
+      <c r="S39" t="str">
+        <v/>
       </c>
       <c r="T39">
         <v>100</v>
@@ -9649,7 +9649,7 @@
         <v>5985</v>
       </c>
       <c r="O40">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P40">
         <v>5985</v>
@@ -9660,8 +9660,8 @@
       <c r="R40">
         <v>5985</v>
       </c>
-      <c r="S40">
-        <v>5985</v>
+      <c r="S40" t="str">
+        <v/>
       </c>
       <c r="T40">
         <v>100</v>
@@ -9885,7 +9885,7 @@
         <v>5985</v>
       </c>
       <c r="O41">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P41">
         <v>5985</v>
@@ -9896,8 +9896,8 @@
       <c r="R41">
         <v>5985</v>
       </c>
-      <c r="S41">
-        <v>5985</v>
+      <c r="S41" t="str">
+        <v/>
       </c>
       <c r="T41">
         <v>100</v>
@@ -10121,7 +10121,7 @@
         <v>5481</v>
       </c>
       <c r="O42">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P42">
         <v>5481</v>
@@ -10132,8 +10132,8 @@
       <c r="R42">
         <v>5481</v>
       </c>
-      <c r="S42">
-        <v>5481</v>
+      <c r="S42" t="str">
+        <v/>
       </c>
       <c r="T42">
         <v>100</v>
@@ -10357,7 +10357,7 @@
         <v>126000</v>
       </c>
       <c r="O43">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P43">
         <v>126000</v>
@@ -10368,8 +10368,8 @@
       <c r="R43">
         <v>126000</v>
       </c>
-      <c r="S43">
-        <v>126000</v>
+      <c r="S43" t="str">
+        <v/>
       </c>
       <c r="T43">
         <v>100</v>
@@ -10593,7 +10593,7 @@
         <v>420</v>
       </c>
       <c r="O44">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P44">
         <v>420</v>
@@ -10604,8 +10604,8 @@
       <c r="R44">
         <v>420</v>
       </c>
-      <c r="S44">
-        <v>420</v>
+      <c r="S44" t="str">
+        <v/>
       </c>
       <c r="T44">
         <v>100</v>
@@ -10829,7 +10829,7 @@
         <v>1281</v>
       </c>
       <c r="O45">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P45">
         <v>1281</v>
@@ -10840,8 +10840,8 @@
       <c r="R45">
         <v>1281</v>
       </c>
-      <c r="S45">
-        <v>1281</v>
+      <c r="S45" t="str">
+        <v/>
       </c>
       <c r="T45">
         <v>100</v>
@@ -11065,7 +11065,7 @@
         <v>5481</v>
       </c>
       <c r="O46">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P46">
         <v>5481</v>
@@ -11076,8 +11076,8 @@
       <c r="R46">
         <v>5481</v>
       </c>
-      <c r="S46">
-        <v>5481</v>
+      <c r="S46" t="str">
+        <v/>
       </c>
       <c r="T46">
         <v>100</v>

</xml_diff>

<commit_message>
fix(vattu): Dat gia tri mac dinh MA_DUONG_DUNG=3.05 va DUONG_DUNG=dung ngoai khi gen du lieu vat tu y te
</commit_message>
<xml_diff>
--- a/data/File_Import_VTYT_VNPT_HIS_78cot.xlsx
+++ b/data/File_Import_VTYT_VNPT_HIS_78cot.xlsx
@@ -664,10 +664,10 @@
         <v>Cái</v>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L2" t="str">
         <v>Công ty cổ phần Tanaphar</v>
@@ -900,10 +900,10 @@
         <v>Cái</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L3" t="str">
         <v>Công ty cổ phần Tanaphar</v>
@@ -1136,10 +1136,10 @@
         <v>Cái</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L4" t="str">
         <v>Công ty cổ phần Tanaphar</v>
@@ -1372,10 +1372,10 @@
         <v>Cái</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K5" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L5" t="str">
         <v>Công ty cổ phần Tanaphar</v>
@@ -1608,10 +1608,10 @@
         <v>Cái</v>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K6" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L6" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -1844,10 +1844,10 @@
         <v>Cái</v>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K7" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L7" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -2080,10 +2080,10 @@
         <v>Cái</v>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K8" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L8" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -2316,10 +2316,10 @@
         <v>Bộ</v>
       </c>
       <c r="J9" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K9" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L9" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -2552,10 +2552,10 @@
         <v>Cái</v>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K10" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L10" t="str">
         <v>Công ty CP Thiết bị Y tế Vinahankook</v>
@@ -2788,10 +2788,10 @@
         <v>Bộ</v>
       </c>
       <c r="J11" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K11" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L11" t="str">
         <v>Hunan Luzhou Huikang Development Co., Ltd.</v>
@@ -3024,10 +3024,10 @@
         <v>Cái</v>
       </c>
       <c r="J12" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K12" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L12" t="str">
         <v>Công ty CP nhựa Y tế Việt Nam</v>
@@ -3260,10 +3260,10 @@
         <v>Cái</v>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K13" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L13" t="str">
         <v>Công ty CP Thiết bị Y tế Vinahankook</v>
@@ -3496,10 +3496,10 @@
         <v>Cái</v>
       </c>
       <c r="J14" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K14" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L14" t="str">
         <v>Công ty TNHH Công nghệ y tế Perfect Việt Nam</v>
@@ -3732,10 +3732,10 @@
         <v>Cái</v>
       </c>
       <c r="J15" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K15" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L15" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -3968,10 +3968,10 @@
         <v>Cái</v>
       </c>
       <c r="J16" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K16" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L16" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -4204,10 +4204,10 @@
         <v>Cái</v>
       </c>
       <c r="J17" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K17" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L17" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -4440,10 +4440,10 @@
         <v>Cái</v>
       </c>
       <c r="J18" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K18" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L18" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -4676,10 +4676,10 @@
         <v>Cái</v>
       </c>
       <c r="J19" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K19" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L19" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -4912,10 +4912,10 @@
         <v>Cái</v>
       </c>
       <c r="J20" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K20" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L20" t="str">
         <v>B. Braun - Việt Nam</v>
@@ -5148,10 +5148,10 @@
         <v>Cái</v>
       </c>
       <c r="J21" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K21" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L21" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -5384,10 +5384,10 @@
         <v>Cái</v>
       </c>
       <c r="J22" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K22" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L22" t="str">
         <v>Công ty TNHH Vật tư y tế Omiga</v>
@@ -5620,10 +5620,10 @@
         <v>Bộ</v>
       </c>
       <c r="J23" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K23" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L23" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -5856,10 +5856,10 @@
         <v>Cái</v>
       </c>
       <c r="J24" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K24" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L24" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -6092,10 +6092,10 @@
         <v>Cái</v>
       </c>
       <c r="J25" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K25" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L25" t="str">
         <v>B. Braun Medical Industries Sdn. Bhd.</v>
@@ -6328,10 +6328,10 @@
         <v>Cái</v>
       </c>
       <c r="J26" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K26" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L26" t="str">
         <v>Terumo (Philippines) Corporation</v>
@@ -6564,10 +6564,10 @@
         <v>Cái</v>
       </c>
       <c r="J27" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K27" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L27" t="str">
         <v>Delta Med S.p.a</v>
@@ -6800,10 +6800,10 @@
         <v>Cái</v>
       </c>
       <c r="J28" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K28" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L28" t="str">
         <v>Romsons International</v>
@@ -7036,10 +7036,10 @@
         <v>Cái</v>
       </c>
       <c r="J29" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K29" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L29" t="str">
         <v>Zhejiang Renon Medical Instrument Co., Ltd</v>
@@ -7272,10 +7272,10 @@
         <v>Cái</v>
       </c>
       <c r="J30" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K30" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L30" t="str">
         <v>Henso Medical (Hangzhou) Co., Ltd.</v>
@@ -7508,10 +7508,10 @@
         <v>Cái</v>
       </c>
       <c r="J31" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K31" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L31" t="str">
         <v>Henso Medical (Hangzhou) Co., Ltd.</v>
@@ -7744,10 +7744,10 @@
         <v>Cái</v>
       </c>
       <c r="J32" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K32" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L32" t="str">
         <v>Zhejiang Renon Medical Instrument Co., Ltd</v>
@@ -7982,10 +7982,10 @@
         <v>Cái</v>
       </c>
       <c r="J33" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K33" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L33" t="str">
         <v>Henso Medical (Hangzhou) Co., Ltd.</v>
@@ -8218,10 +8218,10 @@
         <v>Cái</v>
       </c>
       <c r="J34" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K34" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L34" t="str">
         <v>Wenzhou K.L.F. Medical Plastics Co., Ltd</v>
@@ -8454,10 +8454,10 @@
         <v>Cái</v>
       </c>
       <c r="J35" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K35" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L35" t="str">
         <v>B. Braun</v>
@@ -8690,10 +8690,10 @@
         <v>Bộ</v>
       </c>
       <c r="J36" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K36" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L36" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -8926,10 +8926,10 @@
         <v>Cái</v>
       </c>
       <c r="J37" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K37" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L37" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -9162,10 +9162,10 @@
         <v>Cái</v>
       </c>
       <c r="J38" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K38" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L38" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -9398,10 +9398,10 @@
         <v>Cái</v>
       </c>
       <c r="J39" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K39" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L39" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -9634,10 +9634,10 @@
         <v>Cái</v>
       </c>
       <c r="J40" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K40" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L40" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -9870,10 +9870,10 @@
         <v>Cái</v>
       </c>
       <c r="J41" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K41" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L41" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -10106,10 +10106,10 @@
         <v>Bộ</v>
       </c>
       <c r="J42" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K42" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L42" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -10342,10 +10342,10 @@
         <v>Chai</v>
       </c>
       <c r="J43" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K43" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L43" t="str">
         <v>Công ty TNHH sản xuất đầu tư thương mại Tân Hương - Việt Nam</v>
@@ -10578,10 +10578,10 @@
         <v>Cái</v>
       </c>
       <c r="J44" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K44" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L44" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -10814,10 +10814,10 @@
         <v>Cái</v>
       </c>
       <c r="J45" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K45" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L45" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -11050,10 +11050,10 @@
         <v>Bộ</v>
       </c>
       <c r="J46" t="str">
-        <v/>
+        <v>dùng ngoài</v>
       </c>
       <c r="K46" t="str">
-        <v/>
+        <v>3.05</v>
       </c>
       <c r="L46" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>

</xml_diff>

<commit_message>
fix(vattu): giu nguyen duong dung trong va mac dinh MA_LOAI la VT cho vat tu y te
</commit_message>
<xml_diff>
--- a/data/File_Import_VTYT_VNPT_HIS_78cot.xlsx
+++ b/data/File_Import_VTYT_VNPT_HIS_78cot.xlsx
@@ -664,10 +664,10 @@
         <v>Cái</v>
       </c>
       <c r="J2" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K2" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L2" t="str">
         <v>Công ty cổ phần Tanaphar</v>
@@ -900,10 +900,10 @@
         <v>Cái</v>
       </c>
       <c r="J3" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K3" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L3" t="str">
         <v>Công ty cổ phần Tanaphar</v>
@@ -1136,10 +1136,10 @@
         <v>Cái</v>
       </c>
       <c r="J4" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K4" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L4" t="str">
         <v>Công ty cổ phần Tanaphar</v>
@@ -1372,10 +1372,10 @@
         <v>Cái</v>
       </c>
       <c r="J5" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K5" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L5" t="str">
         <v>Công ty cổ phần Tanaphar</v>
@@ -1608,10 +1608,10 @@
         <v>Cái</v>
       </c>
       <c r="J6" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K6" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L6" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -1844,10 +1844,10 @@
         <v>Cái</v>
       </c>
       <c r="J7" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K7" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L7" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -2080,10 +2080,10 @@
         <v>Cái</v>
       </c>
       <c r="J8" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K8" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L8" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -2316,10 +2316,10 @@
         <v>Bộ</v>
       </c>
       <c r="J9" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K9" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L9" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -2552,10 +2552,10 @@
         <v>Cái</v>
       </c>
       <c r="J10" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K10" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L10" t="str">
         <v>Công ty CP Thiết bị Y tế Vinahankook</v>
@@ -2788,10 +2788,10 @@
         <v>Bộ</v>
       </c>
       <c r="J11" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K11" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L11" t="str">
         <v>Hunan Luzhou Huikang Development Co., Ltd.</v>
@@ -3024,10 +3024,10 @@
         <v>Cái</v>
       </c>
       <c r="J12" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K12" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L12" t="str">
         <v>Công ty CP nhựa Y tế Việt Nam</v>
@@ -3260,10 +3260,10 @@
         <v>Cái</v>
       </c>
       <c r="J13" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K13" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L13" t="str">
         <v>Công ty CP Thiết bị Y tế Vinahankook</v>
@@ -3496,10 +3496,10 @@
         <v>Cái</v>
       </c>
       <c r="J14" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K14" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L14" t="str">
         <v>Công ty TNHH Công nghệ y tế Perfect Việt Nam</v>
@@ -3732,10 +3732,10 @@
         <v>Cái</v>
       </c>
       <c r="J15" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K15" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L15" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -3968,10 +3968,10 @@
         <v>Cái</v>
       </c>
       <c r="J16" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K16" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L16" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -4204,10 +4204,10 @@
         <v>Cái</v>
       </c>
       <c r="J17" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K17" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L17" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -4440,10 +4440,10 @@
         <v>Cái</v>
       </c>
       <c r="J18" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K18" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L18" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -4676,10 +4676,10 @@
         <v>Cái</v>
       </c>
       <c r="J19" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K19" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L19" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -4912,10 +4912,10 @@
         <v>Cái</v>
       </c>
       <c r="J20" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K20" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L20" t="str">
         <v>B. Braun - Việt Nam</v>
@@ -5148,10 +5148,10 @@
         <v>Cái</v>
       </c>
       <c r="J21" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K21" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L21" t="str">
         <v>Công ty CP Nhựa Y tế Việt Nam</v>
@@ -5384,10 +5384,10 @@
         <v>Cái</v>
       </c>
       <c r="J22" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K22" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L22" t="str">
         <v>Công ty TNHH Vật tư y tế Omiga</v>
@@ -5620,10 +5620,10 @@
         <v>Bộ</v>
       </c>
       <c r="J23" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K23" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L23" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -5856,10 +5856,10 @@
         <v>Cái</v>
       </c>
       <c r="J24" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K24" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L24" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -6092,10 +6092,10 @@
         <v>Cái</v>
       </c>
       <c r="J25" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K25" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L25" t="str">
         <v>B. Braun Medical Industries Sdn. Bhd.</v>
@@ -6328,10 +6328,10 @@
         <v>Cái</v>
       </c>
       <c r="J26" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K26" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L26" t="str">
         <v>Terumo (Philippines) Corporation</v>
@@ -6564,10 +6564,10 @@
         <v>Cái</v>
       </c>
       <c r="J27" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K27" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L27" t="str">
         <v>Delta Med S.p.a</v>
@@ -6800,10 +6800,10 @@
         <v>Cái</v>
       </c>
       <c r="J28" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K28" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L28" t="str">
         <v>Romsons International</v>
@@ -7036,10 +7036,10 @@
         <v>Cái</v>
       </c>
       <c r="J29" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K29" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L29" t="str">
         <v>Zhejiang Renon Medical Instrument Co., Ltd</v>
@@ -7272,10 +7272,10 @@
         <v>Cái</v>
       </c>
       <c r="J30" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K30" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L30" t="str">
         <v>Henso Medical (Hangzhou) Co., Ltd.</v>
@@ -7508,10 +7508,10 @@
         <v>Cái</v>
       </c>
       <c r="J31" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K31" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L31" t="str">
         <v>Henso Medical (Hangzhou) Co., Ltd.</v>
@@ -7744,10 +7744,10 @@
         <v>Cái</v>
       </c>
       <c r="J32" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K32" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L32" t="str">
         <v>Zhejiang Renon Medical Instrument Co., Ltd</v>
@@ -7982,10 +7982,10 @@
         <v>Cái</v>
       </c>
       <c r="J33" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K33" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L33" t="str">
         <v>Henso Medical (Hangzhou) Co., Ltd.</v>
@@ -8218,10 +8218,10 @@
         <v>Cái</v>
       </c>
       <c r="J34" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K34" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L34" t="str">
         <v>Wenzhou K.L.F. Medical Plastics Co., Ltd</v>
@@ -8454,10 +8454,10 @@
         <v>Cái</v>
       </c>
       <c r="J35" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K35" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L35" t="str">
         <v>B. Braun</v>
@@ -8690,10 +8690,10 @@
         <v>Bộ</v>
       </c>
       <c r="J36" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K36" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L36" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -8926,10 +8926,10 @@
         <v>Cái</v>
       </c>
       <c r="J37" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K37" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L37" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -9162,10 +9162,10 @@
         <v>Cái</v>
       </c>
       <c r="J38" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K38" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L38" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -9398,10 +9398,10 @@
         <v>Cái</v>
       </c>
       <c r="J39" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K39" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L39" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -9634,10 +9634,10 @@
         <v>Cái</v>
       </c>
       <c r="J40" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K40" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L40" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -9870,10 +9870,10 @@
         <v>Cái</v>
       </c>
       <c r="J41" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K41" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L41" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -10106,10 +10106,10 @@
         <v>Bộ</v>
       </c>
       <c r="J42" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K42" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L42" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -10342,10 +10342,10 @@
         <v>Chai</v>
       </c>
       <c r="J43" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K43" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L43" t="str">
         <v>Công ty TNHH sản xuất đầu tư thương mại Tân Hương - Việt Nam</v>
@@ -10578,10 +10578,10 @@
         <v>Cái</v>
       </c>
       <c r="J44" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K44" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L44" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -10814,10 +10814,10 @@
         <v>Cái</v>
       </c>
       <c r="J45" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K45" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L45" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>
@@ -11050,10 +11050,10 @@
         <v>Bộ</v>
       </c>
       <c r="J46" t="str">
-        <v>dùng ngoài</v>
+        <v/>
       </c>
       <c r="K46" t="str">
-        <v>3.05</v>
+        <v/>
       </c>
       <c r="L46" t="str">
         <v>Công ty CP nhựa y tế Việt Nam</v>

</xml_diff>